<commit_message>
fix: refresh 30-function qualification evidence
</commit_message>
<xml_diff>
--- a/demo/workbooks/case_5_supported_formula_demonstration.xlsx
+++ b/demo/workbooks/case_5_supported_formula_demonstration.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="397" uniqueCount="247">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="285">
   <si>
     <t xml:space="preserve">Case 5: supported formula demonstration</t>
   </si>
@@ -367,6 +367,54 @@
     <t xml:space="preserve">Outputs!C29</t>
   </si>
   <si>
+    <t xml:space="preserve">FML-027</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Leap-day Excel serial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DATE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Outputs!C30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FML-028</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Month-end date shift</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EDATE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Outputs!C31</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FML-029</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inclusive working days</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NETWORKDAYS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Outputs!C32</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FML-030</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Leap-year actual/365 fraction</t>
+  </si>
+  <si>
+    <t xml:space="preserve">YEARFRAC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Outputs!C33</t>
+  </si>
+  <si>
     <t xml:space="preserve">Supported formula calculations</t>
   </si>
   <si>
@@ -460,6 +508,18 @@
     <t xml:space="preserve">Retrieves a numeric exact-match factor with XLOOKUP.</t>
   </si>
   <si>
+    <t xml:space="preserve">Constructs the 2024 leap day as an Excel serial date.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shifts January month-end to the 2024 leap day.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Counts Monday-to-Friday working days in an inclusive calendar week.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Measures the 2024 leap year using the actual/365 convention.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Synthetic portfolio inputs</t>
   </si>
   <si>
@@ -637,6 +697,60 @@
     <t xml:space="preserve">Scenario 3 factor</t>
   </si>
   <si>
+    <t xml:space="preserve">Date start year</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DATE, EDATE, NETWORKDAYS and YEARFRAC controls</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Leap-day month</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DATE control</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Leap-day number</t>
+  </si>
+  <si>
+    <t xml:space="preserve">January month</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EDATE, NETWORKDAYS and YEARFRAC controls</t>
+  </si>
+  <si>
+    <t xml:space="preserve">January month-end day</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EDATE control</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Whole-month shift</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Period start day</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NETWORKDAYS and YEARFRAC controls</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Period end day</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NETWORKDAYS control</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Date end year</t>
+  </si>
+  <si>
+    <t xml:space="preserve">YEARFRAC control</t>
+  </si>
+  <si>
+    <t xml:space="preserve">YEARFRAC basis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Actual/365 convention</t>
+  </si>
+  <si>
     <t xml:space="preserve">Synthetic product lookup</t>
   </si>
   <si>
@@ -682,7 +796,7 @@
     <t xml:space="preserve">Scope</t>
   </si>
   <si>
-    <t xml:space="preserve">All 26 functions declared supported by the production formula catalogue.</t>
+    <t xml:space="preserve">All 30 functions declared supported by the production formula catalogue.</t>
   </si>
   <si>
     <t xml:space="preserve">Synthetic data</t>
@@ -700,7 +814,7 @@
     <t xml:space="preserve">Gate 2 selection</t>
   </si>
   <si>
-    <t xml:space="preserve">Select Outputs!C4:C29 as the authoritative outputs.</t>
+    <t xml:space="preserve">Select Outputs!C4:C33 as the authoritative outputs.</t>
   </si>
   <si>
     <t xml:space="preserve">Gate 3</t>
@@ -727,10 +841,10 @@
     <t xml:space="preserve">Supported calculation population</t>
   </si>
   <si>
-    <t xml:space="preserve">26 complete outputs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Outputs!C4:C29</t>
+    <t xml:space="preserve">30 complete outputs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Outputs!C4:C33</t>
   </si>
   <si>
     <t xml:space="preserve">Internal reconciliation</t>
@@ -773,10 +887,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0.00;[RED]\(#,##0.00\);\-"/>
-    <numFmt numFmtId="166" formatCode="0.00%"/>
+    <numFmt numFmtId="166" formatCode="#,##0"/>
+    <numFmt numFmtId="167" formatCode="0.000000"/>
+    <numFmt numFmtId="168" formatCode="0.00%"/>
   </numFmts>
   <fonts count="11">
     <font>
@@ -1063,7 +1179,7 @@
       <protection locked="true" hidden="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="29">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1092,7 +1208,23 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="8" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1108,7 +1240,7 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="6" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="6" fillId="0" borderId="6" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1124,7 +1256,7 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="9" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="6" fillId="0" borderId="9" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1140,7 +1272,7 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="12" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="6" fillId="0" borderId="12" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1148,7 +1280,7 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="9" fillId="3" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="9" fillId="3" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1411,7 +1543,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:F33"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
@@ -1425,41 +1557,21 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>0</v>
-      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>1</v>
-      </c>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
@@ -2025,6 +2137,90 @@
       </c>
       <c r="F29" s="2" t="s">
         <v>112</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="C30" s="7" t="n">
+        <f aca="false">Calculations!B30</f>
+        <v>45351</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F30" s="2" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="C31" s="7" t="n">
+        <f aca="false">Calculations!B31</f>
+        <v>45351</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F31" s="2" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="C32" s="7" t="n">
+        <f aca="false">Calculations!B32</f>
+        <v>5</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F32" s="2" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="C33" s="8" t="n">
+        <f aca="false">Calculations!B33</f>
+        <v>1.0027397260274</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="E33" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F33" s="2" t="s">
+        <v>128</v>
       </c>
     </row>
   </sheetData>
@@ -2043,7 +2239,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D29"/>
+  <dimension ref="A1:D33"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="36"/>
@@ -2054,51 +2250,39 @@
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>113</v>
-      </c>
+        <v>129</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>114</v>
-      </c>
+        <v>130</v>
+      </c>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>115</v>
+        <v>131</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>116</v>
+        <v>132</v>
       </c>
       <c r="C3" s="4" t="s">
         <v>5</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>117</v>
+        <v>133</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="7" t="n">
+      <c r="B4" s="9" t="n">
         <f aca="false">SUM(Inputs!$F$4:$F$11)</f>
         <v>740000</v>
       </c>
@@ -2106,14 +2290,14 @@
         <v>10</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>118</v>
+        <v>134</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B5" s="7" t="n">
+      <c r="B5" s="9" t="n">
         <f aca="false">ABS(SUM(Inputs!$G$4:$G$11))</f>
         <v>2900</v>
       </c>
@@ -2121,14 +2305,14 @@
         <v>15</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>119</v>
+        <v>135</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B6" s="7" t="n">
+      <c r="B6" s="9" t="n">
         <f aca="false">INT(SUM(Inputs!$E$4:$E$11)/Assumptions!$B$13)</f>
         <v>12</v>
       </c>
@@ -2136,14 +2320,14 @@
         <v>19</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>120</v>
+        <v>136</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B7" s="7" t="n">
+      <c r="B7" s="9" t="n">
         <f aca="false">ROUND(Assumptions!$B$9,Assumptions!$B$6)</f>
         <v>2501</v>
       </c>
@@ -2151,14 +2335,14 @@
         <v>23</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>121</v>
+        <v>137</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B8" s="7" t="n">
+      <c r="B8" s="9" t="n">
         <f aca="false">ROUNDUP(Assumptions!$B$10,Assumptions!$B$7)</f>
         <v>-2500.6</v>
       </c>
@@ -2166,14 +2350,14 @@
         <v>27</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>122</v>
+        <v>138</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B9" s="7" t="n">
+      <c r="B9" s="9" t="n">
         <f aca="false">ROUNDDOWN(Assumptions!$B$10,Assumptions!$B$7)</f>
         <v>-2500.5</v>
       </c>
@@ -2181,14 +2365,14 @@
         <v>31</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>123</v>
+        <v>139</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B10" s="7" t="n">
+      <c r="B10" s="9" t="n">
         <f aca="false">CEILING(Assumptions!$B$9,Assumptions!$B$8)</f>
         <v>2600</v>
       </c>
@@ -2196,14 +2380,14 @@
         <v>35</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>124</v>
+        <v>140</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="B11" s="7" t="n">
+      <c r="B11" s="9" t="n">
         <f aca="false">FLOOR(Assumptions!$B$9,Assumptions!$B$8)</f>
         <v>2500</v>
       </c>
@@ -2211,14 +2395,14 @@
         <v>39</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>125</v>
+        <v>141</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B12" s="7" t="n">
+      <c r="B12" s="9" t="n">
         <f aca="false">SUMIF(Inputs!$B$4:$B$11,Assumptions!$B$4,Inputs!$F$4:$F$11)</f>
         <v>310000</v>
       </c>
@@ -2226,14 +2410,14 @@
         <v>43</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>126</v>
+        <v>142</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="B13" s="7" t="n">
+      <c r="B13" s="9" t="n">
         <f aca="false">SUMIFS(Inputs!$F$4:$F$11,Inputs!$B$4:$B$11,Assumptions!$B$4,Inputs!$C$4:$C$11,Assumptions!$B$5)</f>
         <v>200000</v>
       </c>
@@ -2241,14 +2425,14 @@
         <v>47</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>127</v>
+        <v>143</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B14" s="7" t="n">
+      <c r="B14" s="9" t="n">
         <f aca="false">COUNTIF(Inputs!$B$4:$B$11,Assumptions!$B$4)</f>
         <v>3</v>
       </c>
@@ -2256,14 +2440,14 @@
         <v>51</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>128</v>
+        <v>144</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="B15" s="7" t="n">
+      <c r="B15" s="9" t="n">
         <f aca="false">COUNTIFS(Inputs!$C$4:$C$11,Assumptions!$B$5,Inputs!$D$4:$D$11,Assumptions!$B$14)</f>
         <v>4</v>
       </c>
@@ -2271,14 +2455,14 @@
         <v>55</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>129</v>
+        <v>145</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="B16" s="7" t="n">
+      <c r="B16" s="9" t="n">
         <f aca="false">AVERAGEIF(Inputs!$B$4:$B$11,Assumptions!$B$4,Inputs!$H$4:$H$11)</f>
         <v>2500</v>
       </c>
@@ -2286,14 +2470,14 @@
         <v>59</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>130</v>
+        <v>146</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="B17" s="7" t="n">
+      <c r="B17" s="9" t="n">
         <f aca="false">AVERAGEIFS(Inputs!$F$4:$F$11,Inputs!$C$4:$C$11,Assumptions!$B$5,Inputs!$D$4:$D$11,Assumptions!$B$14)</f>
         <v>87500</v>
       </c>
@@ -2301,14 +2485,14 @@
         <v>63</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>131</v>
+        <v>147</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="B18" s="7" t="n">
+      <c r="B18" s="9" t="n">
         <f aca="false">_xlfn.MINIFS(Inputs!$F$4:$F$11,Inputs!$D$4:$D$11,Assumptions!$B$14)</f>
         <v>70000</v>
       </c>
@@ -2316,14 +2500,14 @@
         <v>67</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>132</v>
+        <v>148</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="B19" s="7" t="n">
+      <c r="B19" s="9" t="n">
         <f aca="false">_xlfn.MAXIFS(Inputs!$F$4:$F$11,Inputs!$D$4:$D$11,Assumptions!$B$14)</f>
         <v>125000</v>
       </c>
@@ -2331,14 +2515,14 @@
         <v>71</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>133</v>
+        <v>149</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="B20" s="7" t="n">
+      <c r="B20" s="9" t="n">
         <f aca="false">IF(Assumptions!$B$15,Inputs!$F$4,IF(Assumptions!$B$16,Inputs!$F$5,Assumptions!$B$11))</f>
         <v>80000</v>
       </c>
@@ -2346,14 +2530,14 @@
         <v>75</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>134</v>
+        <v>150</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="B21" s="7" t="n">
+      <c r="B21" s="9" t="n">
         <f aca="false">VLOOKUP(Assumptions!$B$12,Lookups!$A$4:$B$6,2,FALSE())</f>
         <v>1.08</v>
       </c>
@@ -2361,14 +2545,14 @@
         <v>79</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>135</v>
+        <v>151</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="B22" s="7" t="n">
+      <c r="B22" s="9" t="n">
         <f aca="false">MATCH(Assumptions!$B$12,Lookups!$A$4:$A$6,0)</f>
         <v>2</v>
       </c>
@@ -2376,14 +2560,14 @@
         <v>83</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>136</v>
+        <v>152</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="B23" s="7" t="n">
+      <c r="B23" s="9" t="n">
         <f aca="false">INDEX(Lookups!$B$4:$B$6,MATCH(Assumptions!$B$12,Lookups!$A$4:$A$6,0))</f>
         <v>1.08</v>
       </c>
@@ -2391,14 +2575,14 @@
         <v>87</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>137</v>
+        <v>153</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="B24" s="7" t="n">
+      <c r="B24" s="9" t="n">
         <f aca="false">IF(AND(Assumptions!$B$15,Assumptions!$B$15),1,0)</f>
         <v>1</v>
       </c>
@@ -2406,14 +2590,14 @@
         <v>91</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>138</v>
+        <v>154</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="B25" s="7" t="n">
+      <c r="B25" s="9" t="n">
         <f aca="false">IF(OR(Assumptions!$B$16,Assumptions!$B$15),1,0)</f>
         <v>1</v>
       </c>
@@ -2421,14 +2605,14 @@
         <v>95</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>139</v>
+        <v>155</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="B26" s="7" t="n">
+      <c r="B26" s="9" t="n">
         <f aca="false">SUMPRODUCT(Inputs!$F$4:$F$11,Inputs!$I$4:$I$11)</f>
         <v>760400</v>
       </c>
@@ -2436,14 +2620,14 @@
         <v>99</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>140</v>
+        <v>156</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="B27" s="7" t="n">
+      <c r="B27" s="9" t="n">
         <f aca="false">NPV(Assumptions!$B$17,Lookups!$E$4:$E$7)</f>
         <v>-230.858547913394</v>
       </c>
@@ -2451,14 +2635,14 @@
         <v>103</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>141</v>
+        <v>157</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="B28" s="7" t="n">
+      <c r="B28" s="9" t="n">
         <f aca="false">CHOOSE(2,Assumptions!$B$18,Assumptions!$B$19,Assumptions!$B$20)</f>
         <v>1.08</v>
       </c>
@@ -2466,14 +2650,14 @@
         <v>107</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>142</v>
+        <v>158</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="B29" s="7" t="n">
+      <c r="B29" s="9" t="n">
         <f aca="false">_xlfn.XLOOKUP(Assumptions!$B$12,Lookups!$A$4:$A$6,Lookups!$B$4:$B$6,,0,1)</f>
         <v>1.08</v>
       </c>
@@ -2481,7 +2665,67 @@
         <v>111</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>143</v>
+        <v>159</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="B30" s="10" t="n">
+        <f aca="false">DATE(Assumptions!$B$21,Assumptions!$B$22,Assumptions!$B$23)</f>
+        <v>45351</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="B31" s="10" t="n">
+        <f aca="false">EDATE(DATE(Assumptions!$B$21,Assumptions!$B$24,Assumptions!$B$25),Assumptions!$B$26)</f>
+        <v>45351</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="B32" s="10" t="n">
+        <f aca="false">NETWORKDAYS(DATE(Assumptions!$B$21,Assumptions!$B$24,Assumptions!$B$27),DATE(Assumptions!$B$21,Assumptions!$B$24,Assumptions!$B$28))</f>
+        <v>5</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="B33" s="11" t="n">
+        <f aca="false">YEARFRAC(DATE(Assumptions!$B$21,Assumptions!$B$24,Assumptions!$B$27),DATE(Assumptions!$B$29,Assumptions!$B$24,Assumptions!$B$27),Assumptions!$B$30)</f>
+        <v>1.0027397260274</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>163</v>
       </c>
     </row>
   </sheetData>
@@ -2511,312 +2755,280 @@
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>144</v>
-      </c>
+        <v>164</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>145</v>
-      </c>
+        <v>165</v>
+      </c>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>146</v>
+        <v>166</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>147</v>
+        <v>167</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>148</v>
+        <v>168</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>149</v>
+        <v>169</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>150</v>
+        <v>170</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>151</v>
+        <v>171</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>152</v>
+        <v>172</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>153</v>
+        <v>173</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>154</v>
+        <v>174</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="8" t="s">
-        <v>155</v>
-      </c>
-      <c r="B4" s="9" t="s">
-        <v>156</v>
-      </c>
-      <c r="C4" s="9" t="s">
-        <v>157</v>
-      </c>
-      <c r="D4" s="9" t="s">
-        <v>149</v>
-      </c>
-      <c r="E4" s="10" t="n">
+      <c r="A4" s="12" t="s">
+        <v>175</v>
+      </c>
+      <c r="B4" s="13" t="s">
+        <v>176</v>
+      </c>
+      <c r="C4" s="13" t="s">
+        <v>177</v>
+      </c>
+      <c r="D4" s="13" t="s">
+        <v>169</v>
+      </c>
+      <c r="E4" s="14" t="n">
         <v>120000</v>
       </c>
-      <c r="F4" s="10" t="n">
+      <c r="F4" s="14" t="n">
         <v>80000</v>
       </c>
-      <c r="G4" s="10" t="n">
+      <c r="G4" s="14" t="n">
         <v>-2500</v>
       </c>
-      <c r="H4" s="10"/>
-      <c r="I4" s="11" t="n">
+      <c r="H4" s="14"/>
+      <c r="I4" s="15" t="n">
         <v>0.9</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="12" t="s">
-        <v>158</v>
-      </c>
-      <c r="B5" s="13" t="s">
-        <v>159</v>
-      </c>
-      <c r="C5" s="13" t="s">
-        <v>160</v>
-      </c>
-      <c r="D5" s="13" t="s">
-        <v>149</v>
-      </c>
-      <c r="E5" s="14" t="n">
+      <c r="A5" s="16" t="s">
+        <v>178</v>
+      </c>
+      <c r="B5" s="17" t="s">
+        <v>179</v>
+      </c>
+      <c r="C5" s="17" t="s">
+        <v>180</v>
+      </c>
+      <c r="D5" s="17" t="s">
+        <v>169</v>
+      </c>
+      <c r="E5" s="18" t="n">
         <v>200000</v>
       </c>
-      <c r="F5" s="14" t="n">
+      <c r="F5" s="18" t="n">
         <v>110000</v>
       </c>
-      <c r="G5" s="14" t="n">
+      <c r="G5" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="H5" s="14" t="n">
+      <c r="H5" s="18" t="n">
         <v>5000</v>
       </c>
-      <c r="I5" s="15" t="n">
+      <c r="I5" s="19" t="n">
         <v>1.05</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="12" t="s">
-        <v>161</v>
-      </c>
-      <c r="B6" s="13" t="s">
-        <v>162</v>
-      </c>
-      <c r="C6" s="13" t="s">
-        <v>157</v>
-      </c>
-      <c r="D6" s="13" t="s">
-        <v>163</v>
-      </c>
-      <c r="E6" s="14" t="n">
+      <c r="A6" s="16" t="s">
+        <v>181</v>
+      </c>
+      <c r="B6" s="17" t="s">
+        <v>182</v>
+      </c>
+      <c r="C6" s="17" t="s">
+        <v>177</v>
+      </c>
+      <c r="D6" s="17" t="s">
+        <v>183</v>
+      </c>
+      <c r="E6" s="18" t="n">
         <v>150000</v>
       </c>
-      <c r="F6" s="14" t="n">
+      <c r="F6" s="18" t="n">
         <v>90000</v>
       </c>
-      <c r="G6" s="14" t="n">
+      <c r="G6" s="18" t="n">
         <v>1800</v>
       </c>
-      <c r="H6" s="14"/>
-      <c r="I6" s="15" t="n">
+      <c r="H6" s="18"/>
+      <c r="I6" s="19" t="n">
         <v>1.1</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="12" t="s">
-        <v>164</v>
-      </c>
-      <c r="B7" s="13" t="s">
-        <v>156</v>
-      </c>
-      <c r="C7" s="13" t="s">
-        <v>157</v>
-      </c>
-      <c r="D7" s="13" t="s">
-        <v>149</v>
-      </c>
-      <c r="E7" s="14" t="n">
+      <c r="A7" s="16" t="s">
+        <v>184</v>
+      </c>
+      <c r="B7" s="17" t="s">
+        <v>176</v>
+      </c>
+      <c r="C7" s="17" t="s">
+        <v>177</v>
+      </c>
+      <c r="D7" s="17" t="s">
+        <v>169</v>
+      </c>
+      <c r="E7" s="18" t="n">
         <v>130000</v>
       </c>
-      <c r="F7" s="14" t="n">
+      <c r="F7" s="18" t="n">
         <v>70000</v>
       </c>
-      <c r="G7" s="14" t="n">
+      <c r="G7" s="18" t="n">
         <v>-1200</v>
       </c>
-      <c r="H7" s="14" t="n">
+      <c r="H7" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="I7" s="15" t="n">
+      <c r="I7" s="19" t="n">
         <v>0.95</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="12" t="s">
-        <v>165</v>
-      </c>
-      <c r="B8" s="13" t="s">
-        <v>159</v>
-      </c>
-      <c r="C8" s="13" t="s">
-        <v>157</v>
-      </c>
-      <c r="D8" s="13" t="s">
-        <v>149</v>
-      </c>
-      <c r="E8" s="14" t="n">
+      <c r="A8" s="16" t="s">
+        <v>185</v>
+      </c>
+      <c r="B8" s="17" t="s">
+        <v>179</v>
+      </c>
+      <c r="C8" s="17" t="s">
+        <v>177</v>
+      </c>
+      <c r="D8" s="17" t="s">
+        <v>169</v>
+      </c>
+      <c r="E8" s="18" t="n">
         <v>175000</v>
       </c>
-      <c r="F8" s="14" t="n">
+      <c r="F8" s="18" t="n">
         <v>95000</v>
       </c>
-      <c r="G8" s="14" t="n">
+      <c r="G8" s="18" t="n">
         <v>900</v>
       </c>
-      <c r="H8" s="14" t="n">
+      <c r="H8" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="I8" s="15" t="n">
+      <c r="I8" s="19" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="12" t="s">
-        <v>166</v>
-      </c>
-      <c r="B9" s="13" t="s">
-        <v>162</v>
-      </c>
-      <c r="C9" s="13" t="s">
-        <v>160</v>
-      </c>
-      <c r="D9" s="13" t="s">
-        <v>149</v>
-      </c>
-      <c r="E9" s="14" t="n">
+      <c r="A9" s="16" t="s">
+        <v>186</v>
+      </c>
+      <c r="B9" s="17" t="s">
+        <v>182</v>
+      </c>
+      <c r="C9" s="17" t="s">
+        <v>180</v>
+      </c>
+      <c r="D9" s="17" t="s">
+        <v>169</v>
+      </c>
+      <c r="E9" s="18" t="n">
         <v>220000</v>
       </c>
-      <c r="F9" s="14" t="n">
+      <c r="F9" s="18" t="n">
         <v>125000</v>
       </c>
-      <c r="G9" s="14" t="n">
+      <c r="G9" s="18" t="n">
         <v>-3000</v>
       </c>
-      <c r="H9" s="14"/>
-      <c r="I9" s="15" t="n">
+      <c r="H9" s="18"/>
+      <c r="I9" s="19" t="n">
         <v>1.15</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="12" t="s">
-        <v>167</v>
-      </c>
-      <c r="B10" s="13" t="s">
-        <v>156</v>
-      </c>
-      <c r="C10" s="13" t="s">
-        <v>160</v>
-      </c>
-      <c r="D10" s="13" t="s">
-        <v>163</v>
-      </c>
-      <c r="E10" s="14" t="n">
+      <c r="A10" s="16" t="s">
+        <v>187</v>
+      </c>
+      <c r="B10" s="17" t="s">
+        <v>176</v>
+      </c>
+      <c r="C10" s="17" t="s">
+        <v>180</v>
+      </c>
+      <c r="D10" s="17" t="s">
+        <v>183</v>
+      </c>
+      <c r="E10" s="18" t="n">
         <v>100000</v>
       </c>
-      <c r="F10" s="14" t="n">
+      <c r="F10" s="18" t="n">
         <v>65000</v>
       </c>
-      <c r="G10" s="14" t="n">
+      <c r="G10" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="H10" s="14" t="n">
+      <c r="H10" s="18" t="n">
         <v>2500</v>
       </c>
-      <c r="I10" s="15" t="n">
+      <c r="I10" s="19" t="n">
         <v>0.85</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="16" t="s">
-        <v>168</v>
-      </c>
-      <c r="B11" s="17" t="s">
-        <v>159</v>
-      </c>
-      <c r="C11" s="17" t="s">
-        <v>157</v>
-      </c>
-      <c r="D11" s="17" t="s">
-        <v>149</v>
-      </c>
-      <c r="E11" s="18" t="n">
+      <c r="A11" s="20" t="s">
+        <v>188</v>
+      </c>
+      <c r="B11" s="21" t="s">
+        <v>179</v>
+      </c>
+      <c r="C11" s="21" t="s">
+        <v>177</v>
+      </c>
+      <c r="D11" s="21" t="s">
+        <v>169</v>
+      </c>
+      <c r="E11" s="22" t="n">
         <v>190000</v>
       </c>
-      <c r="F11" s="18" t="n">
+      <c r="F11" s="22" t="n">
         <v>105000</v>
       </c>
-      <c r="G11" s="18" t="n">
+      <c r="G11" s="22" t="n">
         <v>1100</v>
       </c>
-      <c r="H11" s="18"/>
-      <c r="I11" s="19" t="n">
+      <c r="H11" s="22"/>
+      <c r="I11" s="23" t="n">
         <v>1.08</v>
       </c>
     </row>
@@ -2836,7 +3048,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C30"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="31"/>
@@ -2846,14 +3058,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>169</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>169</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>169</v>
-      </c>
+        <v>189</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2"/>
@@ -2862,119 +3070,119 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>170</v>
+        <v>190</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>171</v>
+        <v>191</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>172</v>
+        <v>192</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="B4" s="20" t="s">
-        <v>159</v>
+        <v>193</v>
+      </c>
+      <c r="B4" s="24" t="s">
+        <v>179</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>174</v>
+        <v>194</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>175</v>
-      </c>
-      <c r="B5" s="20" t="s">
-        <v>157</v>
+        <v>195</v>
+      </c>
+      <c r="B5" s="24" t="s">
+        <v>177</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>176</v>
+        <v>196</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="B6" s="20" t="n">
+        <v>197</v>
+      </c>
+      <c r="B6" s="24" t="n">
         <v>0</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>178</v>
+        <v>198</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>179</v>
-      </c>
-      <c r="B7" s="20" t="n">
+        <v>199</v>
+      </c>
+      <c r="B7" s="24" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>180</v>
+        <v>200</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>181</v>
-      </c>
-      <c r="B8" s="20" t="n">
+        <v>201</v>
+      </c>
+      <c r="B8" s="24" t="n">
         <v>100</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>182</v>
+        <v>202</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>183</v>
-      </c>
-      <c r="B9" s="20" t="n">
+        <v>203</v>
+      </c>
+      <c r="B9" s="24" t="n">
         <v>2500.5</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>184</v>
+        <v>204</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>185</v>
-      </c>
-      <c r="B10" s="20" t="n">
+        <v>205</v>
+      </c>
+      <c r="B10" s="24" t="n">
         <v>-2500.51</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>186</v>
+        <v>206</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>187</v>
-      </c>
-      <c r="B11" s="20" t="n">
+        <v>207</v>
+      </c>
+      <c r="B11" s="24" t="n">
         <v>0</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>188</v>
+        <v>208</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>189</v>
-      </c>
-      <c r="B12" s="20" t="s">
-        <v>159</v>
+        <v>209</v>
+      </c>
+      <c r="B12" s="24" t="s">
+        <v>179</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>190</v>
+        <v>210</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>191</v>
-      </c>
-      <c r="B13" s="20" t="n">
+        <v>211</v>
+      </c>
+      <c r="B13" s="24" t="n">
         <v>100000</v>
       </c>
       <c r="C13" s="2" t="s">
@@ -2983,81 +3191,191 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>192</v>
-      </c>
-      <c r="B14" s="20" t="s">
-        <v>149</v>
+        <v>212</v>
+      </c>
+      <c r="B14" s="24" t="s">
+        <v>169</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>193</v>
+        <v>213</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>194</v>
-      </c>
-      <c r="B15" s="20" t="b">
+        <v>214</v>
+      </c>
+      <c r="B15" s="24" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>195</v>
+        <v>215</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>196</v>
-      </c>
-      <c r="B16" s="20" t="b">
+        <v>216</v>
+      </c>
+      <c r="B16" s="24" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>195</v>
+        <v>215</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="B17" s="21" t="n">
+        <v>217</v>
+      </c>
+      <c r="B17" s="25" t="n">
         <v>0.1</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>198</v>
+        <v>218</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="B18" s="21" t="n">
+        <v>219</v>
+      </c>
+      <c r="B18" s="25" t="n">
         <v>0.95</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>200</v>
+        <v>220</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="B19" s="21" t="n">
+        <v>221</v>
+      </c>
+      <c r="B19" s="25" t="n">
         <v>1.08</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>200</v>
+        <v>220</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>202</v>
-      </c>
-      <c r="B20" s="21" t="n">
+        <v>222</v>
+      </c>
+      <c r="B20" s="25" t="n">
         <v>1.15</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>200</v>
+        <v>220</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="B21" s="24" t="n">
+        <v>2024</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="B22" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="B23" s="24" t="n">
+        <v>29</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="B24" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="B25" s="24" t="n">
+        <v>31</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="B26" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="B27" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="B28" s="24" t="n">
+        <v>7</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="B29" s="24" t="n">
+        <v>2025</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="B30" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>240</v>
       </c>
     </row>
   </sheetData>
@@ -3087,14 +3405,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>203</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>203</v>
-      </c>
+        <v>241</v>
+      </c>
+      <c r="B1" s="1"/>
       <c r="C1" s="2"/>
       <c r="D1" s="2" t="s">
-        <v>204</v>
+        <v>242</v>
       </c>
       <c r="E1" s="2"/>
     </row>
@@ -3107,24 +3423,24 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>147</v>
+        <v>167</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>205</v>
+        <v>243</v>
       </c>
       <c r="C3" s="2"/>
       <c r="D3" s="2" t="s">
-        <v>206</v>
+        <v>244</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>207</v>
+        <v>245</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>156</v>
-      </c>
-      <c r="B4" s="20" t="n">
+        <v>176</v>
+      </c>
+      <c r="B4" s="24" t="n">
         <v>1.12</v>
       </c>
       <c r="C4" s="2"/>
@@ -3137,9 +3453,9 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>159</v>
-      </c>
-      <c r="B5" s="20" t="n">
+        <v>179</v>
+      </c>
+      <c r="B5" s="24" t="n">
         <v>1.08</v>
       </c>
       <c r="C5" s="2"/>
@@ -3152,9 +3468,9 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>162</v>
-      </c>
-      <c r="B6" s="20" t="n">
+        <v>182</v>
+      </c>
+      <c r="B6" s="24" t="n">
         <v>1.18</v>
       </c>
       <c r="C6" s="2"/>
@@ -3202,59 +3518,51 @@
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>208</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>208</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>208</v>
-      </c>
+        <v>246</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>209</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>209</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>209</v>
-      </c>
+        <v>247</v>
+      </c>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>210</v>
+        <v>248</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>211</v>
+        <v>249</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>212</v>
+        <v>250</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>213</v>
-      </c>
-      <c r="B4" s="22" t="n">
+        <v>251</v>
+      </c>
+      <c r="B4" s="26" t="n">
         <f aca="false">VLOOKUP(Assumptions!$B$12,Lookups!$A$4:$B$6,2,TRUE())</f>
         <v>1.08</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>214</v>
+        <v>252</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>215</v>
-      </c>
-      <c r="B5" s="23" t="n">
+        <v>253</v>
+      </c>
+      <c r="B5" s="27" t="n">
         <f aca="true">OFFSET(Inputs!$F$4,1,0)</f>
         <v>110000</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>214</v>
+        <v>252</v>
       </c>
     </row>
   </sheetData>
@@ -3283,14 +3591,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>216</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>216</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>216</v>
-      </c>
+        <v>254</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2"/>
@@ -3298,56 +3602,56 @@
       <c r="C2" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="24" t="s">
-        <v>217</v>
+      <c r="A3" s="28" t="s">
+        <v>255</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>218</v>
+        <v>256</v>
       </c>
       <c r="C3" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="24" t="s">
-        <v>219</v>
+      <c r="A4" s="28" t="s">
+        <v>257</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>220</v>
+        <v>258</v>
       </c>
       <c r="C4" s="2"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="24" t="s">
-        <v>221</v>
+      <c r="A5" s="28" t="s">
+        <v>259</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>222</v>
+        <v>260</v>
       </c>
       <c r="C5" s="2"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="24" t="s">
-        <v>223</v>
+      <c r="A6" s="28" t="s">
+        <v>261</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>224</v>
+        <v>262</v>
       </c>
       <c r="C6" s="2"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="24" t="s">
-        <v>225</v>
+      <c r="A7" s="28" t="s">
+        <v>263</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>226</v>
+        <v>264</v>
       </c>
       <c r="C7" s="2"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="24" t="s">
-        <v>227</v>
+      <c r="A8" s="28" t="s">
+        <v>265</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>228</v>
+        <v>266</v>
       </c>
       <c r="C8" s="2"/>
     </row>
@@ -3358,68 +3662,68 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>229</v>
+        <v>267</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>230</v>
+        <v>268</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>231</v>
+        <v>269</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>232</v>
+        <v>270</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>233</v>
+        <v>271</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>234</v>
+        <v>272</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>235</v>
+        <v>273</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>236</v>
+        <v>274</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>237</v>
+        <v>275</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>238</v>
+        <v>276</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>239</v>
+        <v>277</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>240</v>
+        <v>278</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>241</v>
+        <v>279</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>242</v>
+        <v>280</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>243</v>
+        <v>281</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>244</v>
+        <v>282</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>245</v>
+        <v>283</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>246</v>
+        <v>284</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add MAX/MIN formulas and #CALC! error recognition
Adds MAX/MIN as variadic aggregation functions (blank/non-numeric cells
excluded from consideration rather than treated as 0, matching Excel's
own MAX/MIN semantics, distinct from SUM's blank-as-zero convention).
Regenerates the qualification workbook and Case 5's real-workbook
evidence against the live 32-function catalogue, which incidentally
closes the pre-existing Group J qualification gap.

Also adds #CALC! (the dynamic-array-era error) to the parser's
recognized error-value set alongside the seven classic Excel errors,
so it is classified as error evidence rather than silently read as text.

Corrects docs/competition_one_slide.md's test count against the actual
tagged submission commit's CI run (494 -> 496; the doc's number was a
transcription error against the tool's own CI evidence, not drift).
</commit_message>
<xml_diff>
--- a/demo/workbooks/case_5_supported_formula_demonstration.xlsx
+++ b/demo/workbooks/case_5_supported_formula_demonstration.xlsx
@@ -19,14 +19,14 @@
   <calcPr calcId="191029" calcMode="auto" fullCalcOnLoad="1"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
-      <loext:extCalcPr stringRefSyntax="CalcA1ExcelA1"/>
+      <loext:extCalcPr stringRefSyntax="ExcelA1"/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="285">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="424" uniqueCount="295">
   <si>
     <t xml:space="preserve">Case 5: supported formula demonstration</t>
   </si>
@@ -415,6 +415,30 @@
     <t xml:space="preserve">Outputs!C33</t>
   </si>
   <si>
+    <t xml:space="preserve">FML-031</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maximum claim estimate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MAX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Outputs!C34</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FML-032</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Minimum claim estimate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MIN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Outputs!C35</t>
+  </si>
+  <si>
     <t xml:space="preserve">Supported formula calculations</t>
   </si>
   <si>
@@ -520,6 +544,12 @@
     <t xml:space="preserve">Measures the 2024 leap year using the actual/365 convention.</t>
   </si>
   <si>
+    <t xml:space="preserve">Finds the largest claim estimate across the synthetic portfolio.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Finds the smallest claim estimate across the synthetic portfolio.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Synthetic portfolio inputs</t>
   </si>
   <si>
@@ -796,7 +826,7 @@
     <t xml:space="preserve">Scope</t>
   </si>
   <si>
-    <t xml:space="preserve">All 30 functions declared supported by the production formula catalogue.</t>
+    <t xml:space="preserve">All 32 functions declared supported by the production formula catalogue.</t>
   </si>
   <si>
     <t xml:space="preserve">Synthetic data</t>
@@ -814,7 +844,7 @@
     <t xml:space="preserve">Gate 2 selection</t>
   </si>
   <si>
-    <t xml:space="preserve">Select Outputs!C4:C33 as the authoritative outputs.</t>
+    <t xml:space="preserve">Select Outputs!C4:C35 as the authoritative outputs.</t>
   </si>
   <si>
     <t xml:space="preserve">Gate 3</t>
@@ -841,10 +871,10 @@
     <t xml:space="preserve">Supported calculation population</t>
   </si>
   <si>
-    <t xml:space="preserve">30 complete outputs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Outputs!C4:C33</t>
+    <t xml:space="preserve">32 complete outputs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Outputs!C4:C35</t>
   </si>
   <si>
     <t xml:space="preserve">Internal reconciliation</t>
@@ -892,13 +922,14 @@
     <numFmt numFmtId="165" formatCode="#,##0.00;[RED]\(#,##0.00\);\-"/>
     <numFmt numFmtId="166" formatCode="#,##0"/>
     <numFmt numFmtId="167" formatCode="0.000000"/>
-    <numFmt numFmtId="168" formatCode="0.00%"/>
+    <numFmt numFmtId="168" formatCode="0.00\ %"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="10">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -914,12 +945,6 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <family val="0"/>
-      <charset val="1"/>
     </font>
     <font>
       <b val="true"/>
@@ -1150,7 +1175,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="21">
+  <cellStyleXfs count="20">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1174,137 +1199,140 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="31">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="2" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="3" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="8" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="8" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="4" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="5" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="5" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="6" fillId="0" borderId="6" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="7" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="8" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="8" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="6" fillId="0" borderId="9" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="10" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="11" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="11" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="6" fillId="0" borderId="12" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="3" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="9" fillId="3" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="4" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
-  <cellStyles count="7">
+  <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Comma" xfId="15" builtinId="3"/>
     <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
     <cellStyle name="Currency" xfId="17" builtinId="4"/>
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
-    <cellStyle name="Normal" xfId="20"/>
   </cellStyles>
   <colors>
     <indexedColors>
@@ -1543,684 +1571,726 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F33"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="36"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="1" width="18"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="E3" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="F3" s="6" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="6" t="n">
+      <c r="C4" s="7" t="n">
         <f aca="false">Calculations!B4</f>
         <v>740000</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="F4" s="3" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="6" t="n">
+      <c r="C5" s="7" t="n">
         <f aca="false">Calculations!B5</f>
         <v>2900</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="E5" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="F5" s="3" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="C6" s="6" t="n">
+      <c r="C6" s="7" t="n">
         <f aca="false">Calculations!B6</f>
         <v>12</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="D6" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="E6" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="F6" s="2" t="s">
+      <c r="F6" s="3" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="C7" s="6" t="n">
+      <c r="C7" s="7" t="n">
         <f aca="false">Calculations!B7</f>
         <v>2501</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="D7" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="E7" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="F7" s="2" t="s">
+      <c r="F7" s="3" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C8" s="6" t="n">
+      <c r="C8" s="7" t="n">
         <f aca="false">Calculations!B8</f>
         <v>-2500.6</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="D8" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="E8" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="F8" s="2" t="s">
+      <c r="F8" s="3" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="C9" s="6" t="n">
+      <c r="C9" s="7" t="n">
         <f aca="false">Calculations!B9</f>
         <v>-2500.5</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="D9" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="E9" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="F9" s="2" t="s">
+      <c r="F9" s="3" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="C10" s="6" t="n">
+      <c r="C10" s="7" t="n">
         <f aca="false">Calculations!B10</f>
         <v>2600</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="D10" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="E10" s="2" t="s">
+      <c r="E10" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="F10" s="2" t="s">
+      <c r="F10" s="3" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="C11" s="6" t="n">
+      <c r="C11" s="7" t="n">
         <f aca="false">Calculations!B11</f>
         <v>2500</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="D11" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="E11" s="2" t="s">
+      <c r="E11" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="F11" s="2" t="s">
+      <c r="F11" s="3" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="C12" s="6" t="n">
+      <c r="C12" s="7" t="n">
         <f aca="false">Calculations!B12</f>
         <v>310000</v>
       </c>
-      <c r="D12" s="2" t="s">
+      <c r="D12" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="E12" s="2" t="s">
+      <c r="E12" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="F12" s="2" t="s">
+      <c r="F12" s="3" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="2" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B13" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="C13" s="6" t="n">
+      <c r="C13" s="7" t="n">
         <f aca="false">Calculations!B13</f>
         <v>200000</v>
       </c>
-      <c r="D13" s="2" t="s">
+      <c r="D13" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="E13" s="2" t="s">
+      <c r="E13" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="F13" s="2" t="s">
+      <c r="F13" s="3" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="2" t="s">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B14" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="C14" s="6" t="n">
+      <c r="C14" s="7" t="n">
         <f aca="false">Calculations!B14</f>
         <v>3</v>
       </c>
-      <c r="D14" s="2" t="s">
+      <c r="D14" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="E14" s="2" t="s">
+      <c r="E14" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="F14" s="2" t="s">
+      <c r="F14" s="3" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="2" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B15" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="C15" s="6" t="n">
+      <c r="C15" s="7" t="n">
         <f aca="false">Calculations!B15</f>
         <v>4</v>
       </c>
-      <c r="D15" s="2" t="s">
+      <c r="D15" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="E15" s="2" t="s">
+      <c r="E15" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="F15" s="2" t="s">
+      <c r="F15" s="3" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="2" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B16" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="C16" s="6" t="n">
+      <c r="C16" s="7" t="n">
         <f aca="false">Calculations!B16</f>
         <v>2500</v>
       </c>
-      <c r="D16" s="2" t="s">
+      <c r="D16" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="E16" s="2" t="s">
+      <c r="E16" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="F16" s="2" t="s">
+      <c r="F16" s="3" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="2" t="s">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="B17" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="C17" s="6" t="n">
+      <c r="C17" s="7" t="n">
         <f aca="false">Calculations!B17</f>
         <v>87500</v>
       </c>
-      <c r="D17" s="2" t="s">
+      <c r="D17" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="E17" s="2" t="s">
+      <c r="E17" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="F17" s="2" t="s">
+      <c r="F17" s="3" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="2" t="s">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="B18" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="C18" s="6" t="n">
+      <c r="C18" s="7" t="n">
         <f aca="false">Calculations!B18</f>
         <v>70000</v>
       </c>
-      <c r="D18" s="2" t="s">
+      <c r="D18" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="E18" s="2" t="s">
+      <c r="E18" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="F18" s="2" t="s">
+      <c r="F18" s="3" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="2" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="B19" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="C19" s="6" t="n">
+      <c r="C19" s="7" t="n">
         <f aca="false">Calculations!B19</f>
         <v>125000</v>
       </c>
-      <c r="D19" s="2" t="s">
+      <c r="D19" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="E19" s="2" t="s">
+      <c r="E19" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="F19" s="2" t="s">
+      <c r="F19" s="3" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="2" t="s">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="B20" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="C20" s="6" t="n">
+      <c r="C20" s="7" t="n">
         <f aca="false">Calculations!B20</f>
         <v>80000</v>
       </c>
-      <c r="D20" s="2" t="s">
+      <c r="D20" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="E20" s="2" t="s">
+      <c r="E20" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="F20" s="2" t="s">
+      <c r="F20" s="3" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="2" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="B21" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="C21" s="6" t="n">
+      <c r="C21" s="7" t="n">
         <f aca="false">Calculations!B21</f>
         <v>1.08</v>
       </c>
-      <c r="D21" s="2" t="s">
+      <c r="D21" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="E21" s="2" t="s">
+      <c r="E21" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="F21" s="2" t="s">
+      <c r="F21" s="3" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="2" t="s">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="B22" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="C22" s="6" t="n">
+      <c r="C22" s="7" t="n">
         <f aca="false">Calculations!B22</f>
         <v>2</v>
       </c>
-      <c r="D22" s="2" t="s">
+      <c r="D22" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="E22" s="2" t="s">
+      <c r="E22" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="F22" s="2" t="s">
+      <c r="F22" s="3" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="2" t="s">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="B23" s="2" t="s">
+      <c r="B23" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="C23" s="6" t="n">
+      <c r="C23" s="7" t="n">
         <f aca="false">Calculations!B23</f>
         <v>1.08</v>
       </c>
-      <c r="D23" s="2" t="s">
+      <c r="D23" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="E23" s="2" t="s">
+      <c r="E23" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="F23" s="2" t="s">
+      <c r="F23" s="3" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="2" t="s">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="B24" s="2" t="s">
+      <c r="B24" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="C24" s="6" t="n">
+      <c r="C24" s="7" t="n">
         <f aca="false">Calculations!B24</f>
         <v>1</v>
       </c>
-      <c r="D24" s="2" t="s">
+      <c r="D24" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="E24" s="2" t="s">
+      <c r="E24" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="F24" s="2" t="s">
+      <c r="F24" s="3" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="2" t="s">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="B25" s="2" t="s">
+      <c r="B25" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="C25" s="6" t="n">
+      <c r="C25" s="7" t="n">
         <f aca="false">Calculations!B25</f>
         <v>1</v>
       </c>
-      <c r="D25" s="2" t="s">
+      <c r="D25" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="E25" s="2" t="s">
+      <c r="E25" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="F25" s="2" t="s">
+      <c r="F25" s="3" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="2" t="s">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="B26" s="2" t="s">
+      <c r="B26" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="C26" s="6" t="n">
+      <c r="C26" s="7" t="n">
         <f aca="false">Calculations!B26</f>
         <v>760400</v>
       </c>
-      <c r="D26" s="2" t="s">
+      <c r="D26" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="E26" s="2" t="s">
+      <c r="E26" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="F26" s="2" t="s">
+      <c r="F26" s="3" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="2" t="s">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="B27" s="2" t="s">
+      <c r="B27" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="C27" s="6" t="n">
+      <c r="C27" s="7" t="n">
         <f aca="false">Calculations!B27</f>
         <v>-230.858547913394</v>
       </c>
-      <c r="D27" s="2" t="s">
+      <c r="D27" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="E27" s="2" t="s">
+      <c r="E27" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="F27" s="2" t="s">
+      <c r="F27" s="3" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="2" t="s">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="B28" s="2" t="s">
+      <c r="B28" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="C28" s="6" t="n">
+      <c r="C28" s="7" t="n">
         <f aca="false">Calculations!B28</f>
         <v>1.08</v>
       </c>
-      <c r="D28" s="2" t="s">
+      <c r="D28" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="E28" s="2" t="s">
+      <c r="E28" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="F28" s="2" t="s">
+      <c r="F28" s="3" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="2" t="s">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="3" t="s">
         <v>109</v>
       </c>
-      <c r="B29" s="2" t="s">
+      <c r="B29" s="3" t="s">
         <v>110</v>
       </c>
-      <c r="C29" s="6" t="n">
+      <c r="C29" s="7" t="n">
         <f aca="false">Calculations!B29</f>
         <v>1.08</v>
       </c>
-      <c r="D29" s="2" t="s">
+      <c r="D29" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="E29" s="2" t="s">
+      <c r="E29" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="F29" s="2" t="s">
+      <c r="F29" s="3" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="2" t="s">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="B30" s="2" t="s">
+      <c r="B30" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="C30" s="7" t="n">
+      <c r="C30" s="8" t="n">
         <f aca="false">Calculations!B30</f>
         <v>45351</v>
       </c>
-      <c r="D30" s="2" t="s">
+      <c r="D30" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="E30" s="2" t="s">
+      <c r="E30" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="F30" s="2" t="s">
+      <c r="F30" s="3" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="2" t="s">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="3" t="s">
         <v>117</v>
       </c>
-      <c r="B31" s="2" t="s">
+      <c r="B31" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="C31" s="7" t="n">
+      <c r="C31" s="8" t="n">
         <f aca="false">Calculations!B31</f>
         <v>45351</v>
       </c>
-      <c r="D31" s="2" t="s">
+      <c r="D31" s="3" t="s">
         <v>119</v>
       </c>
-      <c r="E31" s="2" t="s">
+      <c r="E31" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="F31" s="2" t="s">
+      <c r="F31" s="3" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="2" t="s">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="B32" s="2" t="s">
+      <c r="B32" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="C32" s="7" t="n">
+      <c r="C32" s="8" t="n">
         <f aca="false">Calculations!B32</f>
         <v>5</v>
       </c>
-      <c r="D32" s="2" t="s">
+      <c r="D32" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="E32" s="2" t="s">
+      <c r="E32" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="F32" s="2" t="s">
+      <c r="F32" s="3" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="2" t="s">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="B33" s="2" t="s">
+      <c r="B33" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="C33" s="8" t="n">
+      <c r="C33" s="9" t="n">
         <f aca="false">Calculations!B33</f>
         <v>1.0027397260274</v>
       </c>
-      <c r="D33" s="2" t="s">
+      <c r="D33" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="E33" s="2" t="s">
+      <c r="E33" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="F33" s="2" t="s">
+      <c r="F33" s="3" t="s">
         <v>128</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="B34" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="C34" s="7" t="n">
+        <f aca="false">Calculations!B34</f>
+        <v>125000</v>
+      </c>
+      <c r="D34" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="E34" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F34" s="3" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="C35" s="7" t="n">
+        <f aca="false">Calculations!B35</f>
+        <v>65000</v>
+      </c>
+      <c r="D35" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="E35" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F35" s="3" t="s">
+        <v>136</v>
       </c>
     </row>
   </sheetData>
@@ -2239,493 +2309,523 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D33"/>
+  <dimension ref="A1:D35"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="36"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="62"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="62"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
-        <v>130</v>
-      </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
-        <v>131</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>132</v>
-      </c>
-      <c r="C3" s="4" t="s">
+      <c r="A1" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="C3" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="D3" s="5" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
+      <c r="D3" s="6" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="9" t="n">
+      <c r="B4" s="10" t="n">
         <f aca="false">SUM(Inputs!$F$4:$F$11)</f>
         <v>740000</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D4" s="2" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="s">
+      <c r="D4" s="3" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B5" s="9" t="n">
+      <c r="B5" s="10" t="n">
         <f aca="false">ABS(SUM(Inputs!$G$4:$G$11))</f>
         <v>2900</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="D5" s="2" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="s">
+      <c r="D5" s="3" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="B6" s="9" t="n">
+      <c r="B6" s="10" t="n">
         <f aca="false">INT(SUM(Inputs!$E$4:$E$11)/Assumptions!$B$13)</f>
         <v>12</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="D6" s="2" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="s">
+      <c r="D6" s="3" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B7" s="9" t="n">
+      <c r="B7" s="10" t="n">
         <f aca="false">ROUND(Assumptions!$B$9,Assumptions!$B$6)</f>
         <v>2501</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="D7" s="2" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="s">
+      <c r="D7" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="B8" s="9" t="n">
+      <c r="B8" s="10" t="n">
         <f aca="false">ROUNDUP(Assumptions!$B$10,Assumptions!$B$7)</f>
         <v>-2500.6</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C8" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="D8" s="2" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="s">
+      <c r="D8" s="3" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="B9" s="9" t="n">
+      <c r="B9" s="10" t="n">
         <f aca="false">ROUNDDOWN(Assumptions!$B$10,Assumptions!$B$7)</f>
         <v>-2500.5</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C9" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="D9" s="2" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2" t="s">
+      <c r="D9" s="3" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="B10" s="9" t="n">
+      <c r="B10" s="10" t="n">
         <f aca="false">CEILING(Assumptions!$B$9,Assumptions!$B$8)</f>
         <v>2600</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C10" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="D10" s="2" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2" t="s">
+      <c r="D10" s="3" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="B11" s="9" t="n">
+      <c r="B11" s="10" t="n">
         <f aca="false">FLOOR(Assumptions!$B$9,Assumptions!$B$8)</f>
         <v>2500</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="C11" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="D11" s="2" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2" t="s">
+      <c r="D11" s="3" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="B12" s="9" t="n">
+      <c r="B12" s="10" t="n">
         <f aca="false">SUMIF(Inputs!$B$4:$B$11,Assumptions!$B$4,Inputs!$F$4:$F$11)</f>
         <v>310000</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="C12" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="D12" s="2" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="2" t="s">
+      <c r="D12" s="3" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="B13" s="9" t="n">
+      <c r="B13" s="10" t="n">
         <f aca="false">SUMIFS(Inputs!$F$4:$F$11,Inputs!$B$4:$B$11,Assumptions!$B$4,Inputs!$C$4:$C$11,Assumptions!$B$5)</f>
         <v>200000</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="C13" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="D13" s="2" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="2" t="s">
+      <c r="D13" s="3" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="B14" s="9" t="n">
+      <c r="B14" s="10" t="n">
         <f aca="false">COUNTIF(Inputs!$B$4:$B$11,Assumptions!$B$4)</f>
         <v>3</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="C14" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="D14" s="2" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="2" t="s">
+      <c r="D14" s="3" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="B15" s="9" t="n">
+      <c r="B15" s="10" t="n">
         <f aca="false">COUNTIFS(Inputs!$C$4:$C$11,Assumptions!$B$5,Inputs!$D$4:$D$11,Assumptions!$B$14)</f>
         <v>4</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="C15" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="D15" s="2" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="2" t="s">
+      <c r="D15" s="3" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="B16" s="9" t="n">
+      <c r="B16" s="10" t="n">
         <f aca="false">AVERAGEIF(Inputs!$B$4:$B$11,Assumptions!$B$4,Inputs!$H$4:$H$11)</f>
         <v>2500</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="C16" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="D16" s="2" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="2" t="s">
+      <c r="D16" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="B17" s="9" t="n">
+      <c r="B17" s="10" t="n">
         <f aca="false">AVERAGEIFS(Inputs!$F$4:$F$11,Inputs!$C$4:$C$11,Assumptions!$B$5,Inputs!$D$4:$D$11,Assumptions!$B$14)</f>
         <v>87500</v>
       </c>
-      <c r="C17" s="2" t="s">
+      <c r="C17" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="D17" s="2" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="2" t="s">
+      <c r="D17" s="3" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="B18" s="9" t="n">
+      <c r="B18" s="10" t="n">
         <f aca="false">_xlfn.MINIFS(Inputs!$F$4:$F$11,Inputs!$D$4:$D$11,Assumptions!$B$14)</f>
         <v>70000</v>
       </c>
-      <c r="C18" s="2" t="s">
+      <c r="C18" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="D18" s="2" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="2" t="s">
+      <c r="D18" s="3" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="B19" s="9" t="n">
+      <c r="B19" s="10" t="n">
         <f aca="false">_xlfn.MAXIFS(Inputs!$F$4:$F$11,Inputs!$D$4:$D$11,Assumptions!$B$14)</f>
         <v>125000</v>
       </c>
-      <c r="C19" s="2" t="s">
+      <c r="C19" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="D19" s="2" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="2" t="s">
+      <c r="D19" s="3" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="B20" s="9" t="n">
+      <c r="B20" s="10" t="n">
         <f aca="false">IF(Assumptions!$B$15,Inputs!$F$4,IF(Assumptions!$B$16,Inputs!$F$5,Assumptions!$B$11))</f>
         <v>80000</v>
       </c>
-      <c r="C20" s="2" t="s">
+      <c r="C20" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="D20" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="2" t="s">
+      <c r="D20" s="3" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="B21" s="9" t="n">
+      <c r="B21" s="10" t="n">
         <f aca="false">VLOOKUP(Assumptions!$B$12,Lookups!$A$4:$B$6,2,FALSE())</f>
         <v>1.08</v>
       </c>
-      <c r="C21" s="2" t="s">
+      <c r="C21" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="D21" s="2" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="2" t="s">
+      <c r="D21" s="3" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="B22" s="9" t="n">
+      <c r="B22" s="10" t="n">
         <f aca="false">MATCH(Assumptions!$B$12,Lookups!$A$4:$A$6,0)</f>
         <v>2</v>
       </c>
-      <c r="C22" s="2" t="s">
+      <c r="C22" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="D22" s="2" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="2" t="s">
+      <c r="D22" s="3" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="B23" s="9" t="n">
+      <c r="B23" s="10" t="n">
         <f aca="false">INDEX(Lookups!$B$4:$B$6,MATCH(Assumptions!$B$12,Lookups!$A$4:$A$6,0))</f>
         <v>1.08</v>
       </c>
-      <c r="C23" s="2" t="s">
+      <c r="C23" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="D23" s="2" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="2" t="s">
+      <c r="D23" s="3" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="B24" s="9" t="n">
+      <c r="B24" s="10" t="n">
         <f aca="false">IF(AND(Assumptions!$B$15,Assumptions!$B$15),1,0)</f>
         <v>1</v>
       </c>
-      <c r="C24" s="2" t="s">
+      <c r="C24" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="D24" s="2" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="2" t="s">
+      <c r="D24" s="3" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="B25" s="9" t="n">
+      <c r="B25" s="10" t="n">
         <f aca="false">IF(OR(Assumptions!$B$16,Assumptions!$B$15),1,0)</f>
         <v>1</v>
       </c>
-      <c r="C25" s="2" t="s">
+      <c r="C25" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="D25" s="2" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="2" t="s">
+      <c r="D25" s="3" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="B26" s="9" t="n">
+      <c r="B26" s="10" t="n">
         <f aca="false">SUMPRODUCT(Inputs!$F$4:$F$11,Inputs!$I$4:$I$11)</f>
         <v>760400</v>
       </c>
-      <c r="C26" s="2" t="s">
+      <c r="C26" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="D26" s="2" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="2" t="s">
+      <c r="D26" s="3" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="B27" s="9" t="n">
+      <c r="B27" s="10" t="n">
         <f aca="false">NPV(Assumptions!$B$17,Lookups!$E$4:$E$7)</f>
         <v>-230.858547913394</v>
       </c>
-      <c r="C27" s="2" t="s">
+      <c r="C27" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="D27" s="2" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="2" t="s">
+      <c r="D27" s="3" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="B28" s="9" t="n">
+      <c r="B28" s="10" t="n">
         <f aca="false">CHOOSE(2,Assumptions!$B$18,Assumptions!$B$19,Assumptions!$B$20)</f>
         <v>1.08</v>
       </c>
-      <c r="C28" s="2" t="s">
+      <c r="C28" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="D28" s="2" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="2" t="s">
+      <c r="D28" s="3" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="3" t="s">
         <v>110</v>
       </c>
-      <c r="B29" s="9" t="n">
+      <c r="B29" s="10" t="n">
         <f aca="false">_xlfn.XLOOKUP(Assumptions!$B$12,Lookups!$A$4:$A$6,Lookups!$B$4:$B$6,,0,1)</f>
         <v>1.08</v>
       </c>
-      <c r="C29" s="2" t="s">
+      <c r="C29" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="D29" s="2" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="2" t="s">
+      <c r="D29" s="3" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="B30" s="10" t="n">
+      <c r="B30" s="11" t="n">
         <f aca="false">DATE(Assumptions!$B$21,Assumptions!$B$22,Assumptions!$B$23)</f>
         <v>45351</v>
       </c>
-      <c r="C30" s="2" t="s">
+      <c r="C30" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="D30" s="2" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="2" t="s">
+      <c r="D30" s="3" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="B31" s="10" t="n">
+      <c r="B31" s="11" t="n">
         <f aca="false">EDATE(DATE(Assumptions!$B$21,Assumptions!$B$24,Assumptions!$B$25),Assumptions!$B$26)</f>
         <v>45351</v>
       </c>
-      <c r="C31" s="2" t="s">
+      <c r="C31" s="3" t="s">
         <v>119</v>
       </c>
-      <c r="D31" s="2" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="2" t="s">
+      <c r="D31" s="3" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="B32" s="10" t="n">
+      <c r="B32" s="11" t="n">
         <f aca="false">NETWORKDAYS(DATE(Assumptions!$B$21,Assumptions!$B$24,Assumptions!$B$27),DATE(Assumptions!$B$21,Assumptions!$B$24,Assumptions!$B$28))</f>
         <v>5</v>
       </c>
-      <c r="C32" s="2" t="s">
+      <c r="C32" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="D32" s="2" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="2" t="s">
+      <c r="D32" s="3" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="B33" s="11" t="n">
+      <c r="B33" s="12" t="n">
         <f aca="false">YEARFRAC(DATE(Assumptions!$B$21,Assumptions!$B$24,Assumptions!$B$27),DATE(Assumptions!$B$29,Assumptions!$B$24,Assumptions!$B$27),Assumptions!$B$30)</f>
         <v>1.0027397260274</v>
       </c>
-      <c r="C33" s="2" t="s">
+      <c r="C33" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="D33" s="2" t="s">
-        <v>163</v>
+      <c r="D33" s="3" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="B34" s="10" t="n">
+        <f aca="false">MAX(Inputs!$F$4:$F$11)</f>
+        <v>125000</v>
+      </c>
+      <c r="C34" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="D34" s="3" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="B35" s="10" t="n">
+        <f aca="false">MIN(Inputs!$F$4:$F$11)</f>
+        <v>65000</v>
+      </c>
+      <c r="C35" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="D35" s="3" t="s">
+        <v>173</v>
       </c>
     </row>
   </sheetData>
@@ -2747,288 +2847,288 @@
   <dimension ref="A1:I11"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="1" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="5" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="1" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="5" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="16"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>164</v>
-      </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="2"/>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
-        <v>166</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>167</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>168</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>169</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>170</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>171</v>
-      </c>
-      <c r="G3" s="4" t="s">
-        <v>172</v>
-      </c>
-      <c r="H3" s="5" t="s">
-        <v>173</v>
-      </c>
-      <c r="I3" s="2" t="s">
+      <c r="A1" s="2" t="s">
         <v>174</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="12" t="s">
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="3"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
         <v>175</v>
       </c>
-      <c r="B4" s="13" t="s">
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="C4" s="13" t="s">
+      <c r="B3" s="5" t="s">
         <v>177</v>
       </c>
-      <c r="D4" s="13" t="s">
-        <v>169</v>
-      </c>
-      <c r="E4" s="14" t="n">
+      <c r="C3" s="5" t="s">
+        <v>178</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>179</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>182</v>
+      </c>
+      <c r="H3" s="6" t="s">
+        <v>183</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="13" t="s">
+        <v>185</v>
+      </c>
+      <c r="B4" s="14" t="s">
+        <v>186</v>
+      </c>
+      <c r="C4" s="14" t="s">
+        <v>187</v>
+      </c>
+      <c r="D4" s="14" t="s">
+        <v>179</v>
+      </c>
+      <c r="E4" s="15" t="n">
         <v>120000</v>
       </c>
-      <c r="F4" s="14" t="n">
+      <c r="F4" s="15" t="n">
         <v>80000</v>
       </c>
-      <c r="G4" s="14" t="n">
+      <c r="G4" s="15" t="n">
         <v>-2500</v>
       </c>
-      <c r="H4" s="14"/>
-      <c r="I4" s="15" t="n">
+      <c r="H4" s="15"/>
+      <c r="I4" s="16" t="n">
         <v>0.9</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="16" t="s">
-        <v>178</v>
-      </c>
-      <c r="B5" s="17" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="17" t="s">
+        <v>188</v>
+      </c>
+      <c r="B5" s="18" t="s">
+        <v>189</v>
+      </c>
+      <c r="C5" s="18" t="s">
+        <v>190</v>
+      </c>
+      <c r="D5" s="18" t="s">
         <v>179</v>
       </c>
-      <c r="C5" s="17" t="s">
-        <v>180</v>
-      </c>
-      <c r="D5" s="17" t="s">
-        <v>169</v>
-      </c>
-      <c r="E5" s="18" t="n">
+      <c r="E5" s="19" t="n">
         <v>200000</v>
       </c>
-      <c r="F5" s="18" t="n">
+      <c r="F5" s="19" t="n">
         <v>110000</v>
       </c>
-      <c r="G5" s="18" t="n">
+      <c r="G5" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="H5" s="18" t="n">
+      <c r="H5" s="19" t="n">
         <v>5000</v>
       </c>
-      <c r="I5" s="19" t="n">
+      <c r="I5" s="20" t="n">
         <v>1.05</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="16" t="s">
-        <v>181</v>
-      </c>
-      <c r="B6" s="17" t="s">
-        <v>182</v>
-      </c>
-      <c r="C6" s="17" t="s">
-        <v>177</v>
-      </c>
-      <c r="D6" s="17" t="s">
-        <v>183</v>
-      </c>
-      <c r="E6" s="18" t="n">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="17" t="s">
+        <v>191</v>
+      </c>
+      <c r="B6" s="18" t="s">
+        <v>192</v>
+      </c>
+      <c r="C6" s="18" t="s">
+        <v>187</v>
+      </c>
+      <c r="D6" s="18" t="s">
+        <v>193</v>
+      </c>
+      <c r="E6" s="19" t="n">
         <v>150000</v>
       </c>
-      <c r="F6" s="18" t="n">
+      <c r="F6" s="19" t="n">
         <v>90000</v>
       </c>
-      <c r="G6" s="18" t="n">
+      <c r="G6" s="19" t="n">
         <v>1800</v>
       </c>
-      <c r="H6" s="18"/>
-      <c r="I6" s="19" t="n">
+      <c r="H6" s="19"/>
+      <c r="I6" s="20" t="n">
         <v>1.1</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="16" t="s">
-        <v>184</v>
-      </c>
-      <c r="B7" s="17" t="s">
-        <v>176</v>
-      </c>
-      <c r="C7" s="17" t="s">
-        <v>177</v>
-      </c>
-      <c r="D7" s="17" t="s">
-        <v>169</v>
-      </c>
-      <c r="E7" s="18" t="n">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="17" t="s">
+        <v>194</v>
+      </c>
+      <c r="B7" s="18" t="s">
+        <v>186</v>
+      </c>
+      <c r="C7" s="18" t="s">
+        <v>187</v>
+      </c>
+      <c r="D7" s="18" t="s">
+        <v>179</v>
+      </c>
+      <c r="E7" s="19" t="n">
         <v>130000</v>
       </c>
-      <c r="F7" s="18" t="n">
+      <c r="F7" s="19" t="n">
         <v>70000</v>
       </c>
-      <c r="G7" s="18" t="n">
+      <c r="G7" s="19" t="n">
         <v>-1200</v>
       </c>
-      <c r="H7" s="18" t="n">
+      <c r="H7" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="I7" s="19" t="n">
+      <c r="I7" s="20" t="n">
         <v>0.95</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="16" t="s">
-        <v>185</v>
-      </c>
-      <c r="B8" s="17" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="17" t="s">
+        <v>195</v>
+      </c>
+      <c r="B8" s="18" t="s">
+        <v>189</v>
+      </c>
+      <c r="C8" s="18" t="s">
+        <v>187</v>
+      </c>
+      <c r="D8" s="18" t="s">
         <v>179</v>
       </c>
-      <c r="C8" s="17" t="s">
-        <v>177</v>
-      </c>
-      <c r="D8" s="17" t="s">
-        <v>169</v>
-      </c>
-      <c r="E8" s="18" t="n">
+      <c r="E8" s="19" t="n">
         <v>175000</v>
       </c>
-      <c r="F8" s="18" t="n">
+      <c r="F8" s="19" t="n">
         <v>95000</v>
       </c>
-      <c r="G8" s="18" t="n">
+      <c r="G8" s="19" t="n">
         <v>900</v>
       </c>
-      <c r="H8" s="18" t="n">
+      <c r="H8" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="I8" s="19" t="n">
+      <c r="I8" s="20" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="16" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="17" t="s">
+        <v>196</v>
+      </c>
+      <c r="B9" s="18" t="s">
+        <v>192</v>
+      </c>
+      <c r="C9" s="18" t="s">
+        <v>190</v>
+      </c>
+      <c r="D9" s="18" t="s">
+        <v>179</v>
+      </c>
+      <c r="E9" s="19" t="n">
+        <v>220000</v>
+      </c>
+      <c r="F9" s="19" t="n">
+        <v>125000</v>
+      </c>
+      <c r="G9" s="19" t="n">
+        <v>-3000</v>
+      </c>
+      <c r="H9" s="19"/>
+      <c r="I9" s="20" t="n">
+        <v>1.15</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="17" t="s">
+        <v>197</v>
+      </c>
+      <c r="B10" s="18" t="s">
         <v>186</v>
       </c>
-      <c r="B9" s="17" t="s">
-        <v>182</v>
-      </c>
-      <c r="C9" s="17" t="s">
-        <v>180</v>
-      </c>
-      <c r="D9" s="17" t="s">
-        <v>169</v>
-      </c>
-      <c r="E9" s="18" t="n">
-        <v>220000</v>
-      </c>
-      <c r="F9" s="18" t="n">
-        <v>125000</v>
-      </c>
-      <c r="G9" s="18" t="n">
-        <v>-3000</v>
-      </c>
-      <c r="H9" s="18"/>
-      <c r="I9" s="19" t="n">
-        <v>1.15</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="16" t="s">
+      <c r="C10" s="18" t="s">
+        <v>190</v>
+      </c>
+      <c r="D10" s="18" t="s">
+        <v>193</v>
+      </c>
+      <c r="E10" s="19" t="n">
+        <v>100000</v>
+      </c>
+      <c r="F10" s="19" t="n">
+        <v>65000</v>
+      </c>
+      <c r="G10" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="19" t="n">
+        <v>2500</v>
+      </c>
+      <c r="I10" s="20" t="n">
+        <v>0.85</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="21" t="s">
+        <v>198</v>
+      </c>
+      <c r="B11" s="22" t="s">
+        <v>189</v>
+      </c>
+      <c r="C11" s="22" t="s">
         <v>187</v>
       </c>
-      <c r="B10" s="17" t="s">
-        <v>176</v>
-      </c>
-      <c r="C10" s="17" t="s">
-        <v>180</v>
-      </c>
-      <c r="D10" s="17" t="s">
-        <v>183</v>
-      </c>
-      <c r="E10" s="18" t="n">
-        <v>100000</v>
-      </c>
-      <c r="F10" s="18" t="n">
-        <v>65000</v>
-      </c>
-      <c r="G10" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="H10" s="18" t="n">
-        <v>2500</v>
-      </c>
-      <c r="I10" s="19" t="n">
-        <v>0.85</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="20" t="s">
-        <v>188</v>
-      </c>
-      <c r="B11" s="21" t="s">
+      <c r="D11" s="22" t="s">
         <v>179</v>
       </c>
-      <c r="C11" s="21" t="s">
-        <v>177</v>
-      </c>
-      <c r="D11" s="21" t="s">
-        <v>169</v>
-      </c>
-      <c r="E11" s="22" t="n">
+      <c r="E11" s="23" t="n">
         <v>190000</v>
       </c>
-      <c r="F11" s="22" t="n">
+      <c r="F11" s="23" t="n">
         <v>105000</v>
       </c>
-      <c r="G11" s="22" t="n">
+      <c r="G11" s="23" t="n">
         <v>1100</v>
       </c>
-      <c r="H11" s="22"/>
-      <c r="I11" s="23" t="n">
+      <c r="H11" s="23"/>
+      <c r="I11" s="24" t="n">
         <v>1.08</v>
       </c>
     </row>
@@ -3051,331 +3151,331 @@
   <dimension ref="A1:C30"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="31"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="48"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>201</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="s">
+        <v>203</v>
+      </c>
+      <c r="B4" s="25" t="s">
         <v>189</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2"/>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
-        <v>190</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>191</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
-        <v>193</v>
-      </c>
-      <c r="B4" s="24" t="s">
+      <c r="C4" s="3" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3" t="s">
+        <v>205</v>
+      </c>
+      <c r="B5" s="25" t="s">
+        <v>187</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="3" t="s">
+        <v>207</v>
+      </c>
+      <c r="B6" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="3" t="s">
+        <v>209</v>
+      </c>
+      <c r="B7" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="B8" s="25" t="n">
+        <v>100</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="B9" s="25" t="n">
+        <v>2500.5</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="B10" s="25" t="n">
+        <v>-2500.51</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="3" t="s">
+        <v>217</v>
+      </c>
+      <c r="B11" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="B12" s="25" t="s">
+        <v>189</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="3" t="s">
+        <v>221</v>
+      </c>
+      <c r="B13" s="25" t="n">
+        <v>100000</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="3" t="s">
+        <v>222</v>
+      </c>
+      <c r="B14" s="25" t="s">
         <v>179</v>
       </c>
-      <c r="C4" s="2" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="B5" s="24" t="s">
-        <v>177</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="B6" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="B7" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="B8" s="24" t="n">
-        <v>100</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="s">
-        <v>203</v>
-      </c>
-      <c r="B9" s="24" t="n">
-        <v>2500.5</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2" t="s">
-        <v>205</v>
-      </c>
-      <c r="B10" s="24" t="n">
-        <v>-2500.51</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2" t="s">
-        <v>207</v>
-      </c>
-      <c r="B11" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2" t="s">
-        <v>209</v>
-      </c>
-      <c r="B12" s="24" t="s">
-        <v>179</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="2" t="s">
-        <v>211</v>
-      </c>
-      <c r="B13" s="24" t="n">
-        <v>100000</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="2" t="s">
-        <v>212</v>
-      </c>
-      <c r="B14" s="24" t="s">
-        <v>169</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="2" t="s">
-        <v>214</v>
-      </c>
-      <c r="B15" s="24" t="b">
+      <c r="C14" s="3" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="3" t="s">
+        <v>224</v>
+      </c>
+      <c r="B15" s="26" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="C15" s="2" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="2" t="s">
-        <v>216</v>
-      </c>
-      <c r="B16" s="24" t="b">
+      <c r="C15" s="3" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="3" t="s">
+        <v>226</v>
+      </c>
+      <c r="B16" s="26" t="b">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="C16" s="2" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="2" t="s">
-        <v>217</v>
-      </c>
-      <c r="B17" s="25" t="n">
+      <c r="C16" s="3" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="B17" s="27" t="n">
         <v>0.1</v>
       </c>
-      <c r="C17" s="2" t="s">
-        <v>218</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="2" t="s">
-        <v>219</v>
-      </c>
-      <c r="B18" s="25" t="n">
+      <c r="C17" s="3" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="B18" s="27" t="n">
         <v>0.95</v>
       </c>
-      <c r="C18" s="2" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="2" t="s">
-        <v>221</v>
-      </c>
-      <c r="B19" s="25" t="n">
+      <c r="C18" s="3" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="3" t="s">
+        <v>231</v>
+      </c>
+      <c r="B19" s="27" t="n">
         <v>1.08</v>
       </c>
-      <c r="C19" s="2" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="2" t="s">
-        <v>222</v>
-      </c>
-      <c r="B20" s="25" t="n">
+      <c r="C19" s="3" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="B20" s="27" t="n">
         <v>1.15</v>
       </c>
-      <c r="C20" s="2" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="2" t="s">
-        <v>223</v>
-      </c>
-      <c r="B21" s="24" t="n">
+      <c r="C20" s="3" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="B21" s="25" t="n">
         <v>2024</v>
       </c>
-      <c r="C21" s="2" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="2" t="s">
-        <v>225</v>
-      </c>
-      <c r="B22" s="24" t="n">
+      <c r="C21" s="3" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="B22" s="25" t="n">
         <v>2</v>
       </c>
-      <c r="C22" s="2" t="s">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="2" t="s">
-        <v>227</v>
-      </c>
-      <c r="B23" s="24" t="n">
+      <c r="C22" s="3" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="3" t="s">
+        <v>237</v>
+      </c>
+      <c r="B23" s="25" t="n">
         <v>29</v>
       </c>
-      <c r="C23" s="2" t="s">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="2" t="s">
-        <v>228</v>
-      </c>
-      <c r="B24" s="24" t="n">
+      <c r="C23" s="3" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="3" t="s">
+        <v>238</v>
+      </c>
+      <c r="B24" s="25" t="n">
         <v>1</v>
       </c>
-      <c r="C24" s="2" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="2" t="s">
-        <v>230</v>
-      </c>
-      <c r="B25" s="24" t="n">
+      <c r="C24" s="3" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="3" t="s">
+        <v>240</v>
+      </c>
+      <c r="B25" s="25" t="n">
         <v>31</v>
       </c>
-      <c r="C25" s="2" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="2" t="s">
-        <v>232</v>
-      </c>
-      <c r="B26" s="24" t="n">
+      <c r="C25" s="3" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="3" t="s">
+        <v>242</v>
+      </c>
+      <c r="B26" s="25" t="n">
         <v>1</v>
       </c>
-      <c r="C26" s="2" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="2" t="s">
-        <v>233</v>
-      </c>
-      <c r="B27" s="24" t="n">
+      <c r="C26" s="3" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="3" t="s">
+        <v>243</v>
+      </c>
+      <c r="B27" s="25" t="n">
         <v>1</v>
       </c>
-      <c r="C27" s="2" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="2" t="s">
-        <v>235</v>
-      </c>
-      <c r="B28" s="24" t="n">
+      <c r="C27" s="3" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="3" t="s">
+        <v>245</v>
+      </c>
+      <c r="B28" s="25" t="n">
         <v>7</v>
       </c>
-      <c r="C28" s="2" t="s">
-        <v>236</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="2" t="s">
-        <v>237</v>
-      </c>
-      <c r="B29" s="24" t="n">
+      <c r="C28" s="3" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="B29" s="25" t="n">
         <v>2025</v>
       </c>
-      <c r="C29" s="2" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="2" t="s">
-        <v>239</v>
-      </c>
-      <c r="B30" s="24" t="n">
+      <c r="C29" s="3" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B30" s="25" t="n">
         <v>3</v>
       </c>
-      <c r="C30" s="2" t="s">
-        <v>240</v>
+      <c r="C30" s="3" t="s">
+        <v>250</v>
       </c>
     </row>
   </sheetData>
@@ -3397,98 +3497,98 @@
   <dimension ref="A1:E7"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="22"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>241</v>
-      </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2" t="s">
-        <v>242</v>
-      </c>
-      <c r="E1" s="2"/>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2"/>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
-        <v>167</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>243</v>
-      </c>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2" t="s">
-        <v>244</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="B4" s="24" t="n">
+      <c r="A1" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3" t="s">
+        <v>252</v>
+      </c>
+      <c r="E1" s="3"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3" t="s">
+        <v>254</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="B4" s="25" t="n">
         <v>1.12</v>
       </c>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2" t="n">
+      <c r="C4" s="3"/>
+      <c r="D4" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="E4" s="2" t="n">
+      <c r="E4" s="3" t="n">
         <v>-1000</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="s">
-        <v>179</v>
-      </c>
-      <c r="B5" s="24" t="n">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="B5" s="25" t="n">
         <v>1.08</v>
       </c>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2" t="n">
+      <c r="C5" s="3"/>
+      <c r="D5" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="E5" s="2" t="n">
+      <c r="E5" s="3" t="n">
         <v>300</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="s">
-        <v>182</v>
-      </c>
-      <c r="B6" s="24" t="n">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="B6" s="25" t="n">
         <v>1.18</v>
       </c>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2" t="n">
+      <c r="C6" s="3"/>
+      <c r="D6" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="E6" s="2" t="n">
+      <c r="E6" s="3" t="n">
         <v>300</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2"/>
-      <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2" t="n">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="3"/>
+      <c r="B7" s="3"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="E7" s="2" t="n">
+      <c r="E7" s="3" t="n">
         <v>300</v>
       </c>
     </row>
@@ -3511,58 +3611,58 @@
   <dimension ref="A1:C5"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="28"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>246</v>
-      </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
-        <v>247</v>
-      </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
-        <v>248</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>249</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
-        <v>251</v>
-      </c>
-      <c r="B4" s="26" t="n">
+      <c r="A1" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
+        <v>257</v>
+      </c>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="4" t="s">
+        <v>258</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>259</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="s">
+        <v>261</v>
+      </c>
+      <c r="B4" s="28" t="n">
         <f aca="false">VLOOKUP(Assumptions!$B$12,Lookups!$A$4:$B$6,2,TRUE())</f>
         <v>1.08</v>
       </c>
-      <c r="C4" s="2" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="s">
-        <v>253</v>
-      </c>
-      <c r="B5" s="27" t="n">
+      <c r="C4" s="3" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="B5" s="29" t="n">
         <f aca="true">OFFSET(Inputs!$F$4,1,0)</f>
         <v>110000</v>
       </c>
-      <c r="C5" s="2" t="s">
-        <v>252</v>
+      <c r="C5" s="3" t="s">
+        <v>262</v>
       </c>
     </row>
   </sheetData>
@@ -3584,146 +3684,146 @@
   <dimension ref="A1:C15"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="85"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="85"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="48"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>254</v>
-      </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2"/>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="28" t="s">
-        <v>255</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>256</v>
-      </c>
-      <c r="C3" s="2"/>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="28" t="s">
-        <v>257</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>258</v>
-      </c>
-      <c r="C4" s="2"/>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="28" t="s">
-        <v>259</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>260</v>
-      </c>
-      <c r="C5" s="2"/>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="28" t="s">
-        <v>261</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>262</v>
-      </c>
-      <c r="C6" s="2"/>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="28" t="s">
-        <v>263</v>
-      </c>
-      <c r="B7" s="2" t="s">
+      <c r="A1" s="2" t="s">
         <v>264</v>
       </c>
-      <c r="C7" s="2"/>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="28" t="s">
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="30" t="s">
         <v>265</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B3" s="3" t="s">
         <v>266</v>
       </c>
-      <c r="C8" s="2"/>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2"/>
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="s">
+      <c r="C3" s="3"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="30" t="s">
         <v>267</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B4" s="3" t="s">
         <v>268</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="C4" s="3"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="30" t="s">
         <v>269</v>
       </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2" t="s">
+      <c r="B5" s="3" t="s">
         <v>270</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="C5" s="3"/>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="30" t="s">
         <v>271</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="B6" s="3" t="s">
         <v>272</v>
       </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2" t="s">
+      <c r="C6" s="3"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="30" t="s">
         <v>273</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B7" s="3" t="s">
         <v>274</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="C7" s="3"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="30" t="s">
         <v>275</v>
       </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="2" t="s">
+      <c r="B8" s="3" t="s">
         <v>276</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="C8" s="3"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="3"/>
+      <c r="B9" s="3"/>
+      <c r="C9" s="3"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4" t="s">
         <v>277</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="B10" s="5" t="s">
         <v>278</v>
       </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="2" t="s">
+      <c r="C10" s="6" t="s">
         <v>279</v>
       </c>
-      <c r="B14" s="2" t="s">
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="3" t="s">
         <v>280</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="B11" s="3" t="s">
         <v>281</v>
       </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="2" t="s">
+      <c r="C11" s="3" t="s">
         <v>282</v>
       </c>
-      <c r="B15" s="2" t="s">
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="3" t="s">
         <v>283</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="B12" s="3" t="s">
         <v>284</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="3" t="s">
+        <v>286</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>290</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="3" t="s">
+        <v>292</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>293</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>294</v>
       </c>
     </row>
   </sheetData>

</xml_diff>